<commit_message>
AI auditlog week9 week10
</commit_message>
<xml_diff>
--- a/LeQuangMinh_AIAuditLog_Week8.xlsx
+++ b/LeQuangMinh_AIAuditLog_Week8.xlsx
@@ -512,7 +512,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="14.4" customHeight="1" s="28">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -564,15 +563,26 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>MotoRental Project - Week 8</t>
-        </is>
-      </c>
-    </row>
-    <row r="8"/>
+          <t>Week 8 (Project Documentation &amp; SDS Alignment)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>01/07/2026</t>
+        </is>
+      </c>
+    </row>
     <row r="9" ht="14.4" customHeight="1" s="28">
       <c r="A9" s="1" t="inlineStr">
         <is>
           <t>AI USAGE SUMMARY</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>07/07/2026</t>
         </is>
       </c>
     </row>
@@ -622,11 +632,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="14.4" customHeight="1" s="28">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>AI TOOLS USED</t>
+          <t>1. Completed generation of Software Design Specification (SDS) exactly matching JobTrans styles/themes.
+2. Synchronized database schemas from SQLMOTO.md into the SDS design.
+3. Verified class diagram structures and sequence flows for all UC modules.</t>
         </is>
       </c>
     </row>
@@ -740,7 +751,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22" ht="14.4" customHeight="1" s="28">
       <c r="A22" s="1" t="inlineStr">
         <is>
@@ -844,7 +854,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10" customWidth="1" style="28" min="1" max="1"/>
@@ -913,356 +923,530 @@
       </c>
     </row>
     <row r="4" ht="115.95" customHeight="1" s="28">
-      <c r="A4" s="23" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>001</t>
         </is>
       </c>
-      <c r="B4" s="23" t="inlineStr">
-        <is>
-          <t>PLANNING</t>
-        </is>
-      </c>
-      <c r="C4" s="23" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>PROBLEM-SOLVING</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>Algorithms</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>Thiết kế logic tính phí trả xe muộn (late fee) trong AdminExtensionServlet và TransactionServlet</t>
+        </is>
+      </c>
+      <c r="E4" s="15" t="inlineStr">
+        <is>
+          <t>Đề xuất công thức late fee: số giờ trễ × hourlyRate × penaltyFactor, xử lý edge case dưới 30 phút miễn phí và trường hợp xe hỏng giữa chừng.</t>
+        </is>
+      </c>
+      <c r="F4" s="15" t="inlineStr">
+        <is>
+          <t>AI đề xuất công thức lateFee = max(0, overtimeHours - 0.5) × hourlyRate × penaltyFactor với penaltyFactor mặc định 1.5, thêm enum LateReason (CUSTOMER_FAULT, VEHICLE_ISSUE, WEATHER).</t>
+        </is>
+      </c>
+      <c r="G4" s="15" t="inlineStr">
+        <is>
+          <t>Critical Thinking: Cần phân biệt lý do trả muộn để áp phí khác nhau, không phải mọi trường hợp đều phạt full. Contextualization: Chính sách MotoRental miễn phí 30 phút đầu và giảm 50% phí nếu lỗi xe. Creative Synthesis: Thêm LateReason enum và configurable penaltyFactor theo từng loại lý do. Decision Ownership: Chốt công thức, thêm cột lateReason và lateFeeAmount vào bảng Booking.</t>
+        </is>
+      </c>
+      <c r="H4" s="15" t="inlineStr">
+        <is>
+          <t>LateFeePolicyService.java / AdminExtensionServlet.java / Booking schema update</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="115.95" customHeight="1" s="28">
+      <c r="A5" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>PROBLEM-SOLVING</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
         <is>
           <t>Decomposition</t>
         </is>
       </c>
-      <c r="D4" s="23" t="inlineStr">
-        <is>
-          <t>Phân tích cấu trúc chuẩn của tài liệu SDS để tạo MotoRental_SDS_final.docx đúng format</t>
-        </is>
-      </c>
-      <c r="E4" s="23" t="inlineStr">
-        <is>
-          <t>Yêu cầu AI đọc và phân tích cấu trúc heading của GroupJobTrans_SDS_final.docx (I. Overview → II. Code Designs → mỗi feature gồm a/b/c/d), sau đó mapping sang module của MotoRental.</t>
-        </is>
-      </c>
-      <c r="F4" s="23" t="inlineStr">
-        <is>
-          <t>AI phân tích được 4 cấp heading (H1/H2/H3/H4), xác định 7 nhóm chức năng chính: Authentication, Account, Motorcycle, Booking, Staff Rental, Admin, Support. Đề xuất giữ nguyên pattern a.Class Diagram / b.Class Spec / c.Sequence Diagram / d.DB Queries.</t>
-        </is>
-      </c>
-      <c r="G4" s="23" t="inlineStr">
-        <is>
-          <t>Critical Thinking: Không thể copy 1:1 từ JobTrans vì domain khác nhau — JobTrans có CV/Job/Recruitment, MotoRental có Booking/Extension/GPS. Contextualization: Deadline nộp báo cáo gần, cần tài liệu đủ khung để team điền ảnh UML vào. Creative Synthesis: Dùng Python-docx để auto-generate toàn bộ khung SDS với đúng heading hierarchy, điền sẵn class specs và SQL queries từ source code thực tế. Decision Ownership: Quyết định giữ 32 sub-feature (H3) và 120 H4 headings, để placeholder cho ảnh UML.</t>
-        </is>
-      </c>
-      <c r="H4" s="23" t="inlineStr">
-        <is>
-          <t>MotoRental_SDS_final.docx / generate_sds.py</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="115.95" customHeight="1" s="28">
-      <c r="A5" s="23" t="inlineStr">
-        <is>
-          <t>002</t>
-        </is>
-      </c>
-      <c r="B5" s="23" t="inlineStr">
-        <is>
-          <t>IMPLEMENTATION</t>
-        </is>
-      </c>
-      <c r="C5" s="23" t="inlineStr">
+      <c r="D5" s="15" t="inlineStr">
+        <is>
+          <t>Yêu cầu tạo file SDS (Software Design Specification) kế thừa đúng style, font chữ, màu sắc của tài liệu tham khảo JobTrans thay vì tạo file trắng trơn.</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>Làm thế nào để lấy được style gốc (Heading 1/2/3, màu đỏ đặc trưng, bảng biểu) từ file docx JobTrans sang MotoRental?</t>
+        </is>
+      </c>
+      <c r="F5" s="15" t="inlineStr">
+        <is>
+          <t>AI gợi ý sử dụng thư viện python-docx để load trực tiếp file Group5_JobTrans_SDS_final.docx.docx làm base template, xóa toàn bộ nội dung text cũ đi nhưng giữ nguyên styles.xml và theme, sau đó chèn nội dung của MotoRental vào.</t>
+        </is>
+      </c>
+      <c r="G5" s="15" t="inlineStr">
+        <is>
+          <t>Critical Thinking: Cách này chính xác và tiết kiệm thời gian hơn việc định nghĩa lại từng style thủ công. Contextualization: Form mẫu của khóa SWP391 FPT cần sự đồng nhất. Decision Ownership: Chấp nhận giải pháp, chạy script Python python-docx để gen file mới MotoRental_SDS_v2.docx.</t>
+        </is>
+      </c>
+      <c r="H5" s="15" t="inlineStr">
+        <is>
+          <t>gen_sds_final.py / MotoRental_SDS_v2.docx</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="115.95" customHeight="1" s="28">
+      <c r="A6" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>DECISION-MAKING</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
         <is>
           <t>Pattern Recognition</t>
         </is>
       </c>
-      <c r="D5" s="23" t="inlineStr">
-        <is>
-          <t>Trích xuất và mapping toàn bộ SQL queries từ SQLMOTO.md vào đúng section của SDS</t>
-        </is>
-      </c>
-      <c r="E5" s="23" t="inlineStr">
-        <is>
-          <t>Yêu cầu AI đọc SQLMOTO.md (657 dòng, 25 bảng), xác định các query CRUD thuộc module nào (Booking, Payment, Motorcycle...) và điền vào phần d.Database Queries của từng feature trong SDS.</t>
-        </is>
-      </c>
-      <c r="F5" s="23" t="inlineStr">
-        <is>
-          <t>AI nhận ra pattern: mỗi bảng chính (Booking, Payment, Extension) cần 4 loại query cơ bản INSERT/SELECT/UPDATE/DELETE, gợi ý thêm JOIN query cho các bảng liên kết như Booking Detail ↔ Motorcycle Detail.</t>
-        </is>
-      </c>
-      <c r="G5" s="23" t="inlineStr">
-        <is>
-          <t>Critical Thinking: AI ban đầu dùng tên cột sai (status thay vì StatusBooking, id thay vì BookingID) — cần verify lại từng column name trong SQLMOTO.md. Contextualization: PostgreSQL dùng dấu nháy kép cho tên cột/bảng, khác SQL Server, nên query cần đúng cú pháp. Creative Synthesis: Thêm cả query JOIN phức tạp (Booking + Customer + Account) vào section Staff Rental Management để SDS đầy đủ hơn. Decision Ownership: Chỉ giữ các query đã thực sự có trong codebase (DAO classes), bỏ các query AI tự sinh ra chưa verify.</t>
-        </is>
-      </c>
-      <c r="H5" s="23" t="inlineStr">
-        <is>
-          <t>SQLMOTO.md / BookingDAO.java / PaymentDAO.java</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="115.95" customHeight="1" s="28">
-      <c r="A6" s="23" t="inlineStr">
-        <is>
-          <t>003</t>
-        </is>
-      </c>
-      <c r="B6" s="23" t="inlineStr">
-        <is>
-          <t>VERIFICATION</t>
-        </is>
-      </c>
-      <c r="C6" s="23" t="inlineStr">
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>Cần đồng bộ Use Case descriptions và UI/Database Access từ tài liệu RDS sang SDS cho 7 phân hệ chính.</t>
+        </is>
+      </c>
+      <c r="E6" s="15" t="inlineStr">
+        <is>
+          <t>Nội dung bên RDS đã có đủ Database Access SQL queries và UI descriptions. Liệu có thể bóc tách tự động và đưa sang phần Code Designs của SDS?</t>
+        </is>
+      </c>
+      <c r="F6" s="15" t="inlineStr">
+        <is>
+          <t>AI thực thi script phân tích MotoRental_RDS_final2026_FIXED.docx, bóc tách các đoạn mapping với CSDL và Use case flow. Gợi ý cấu trúc: a. Class Diagram, b. Class Spec, c. Sequence Diagram, d. Database Queries.</t>
+        </is>
+      </c>
+      <c r="G6" s="15" t="inlineStr">
+        <is>
+          <t>Creative Synthesis: Đã tổng hợp chính xác các queries quan trọng (Register, OTP, Payment Webhook). Quyết định tạo placeholder dạng text xám in nghiêng '[Dán ảnh Class Diagram tại đây]' để sau này dễ dán ảnh mà không bị trượt format. Quyết định rất thông minh.</t>
+        </is>
+      </c>
+      <c r="H6" s="15" t="inlineStr">
+        <is>
+          <t>MotoRental_SDS_v2.docx / SQLMOTO.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="115.95" customHeight="1" s="28">
+      <c r="A7" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>CONCEPTUAL-UNDERSTANDING</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="inlineStr">
         <is>
           <t>Abstraction</t>
         </is>
       </c>
-      <c r="D6" s="23" t="inlineStr">
-        <is>
-          <t>Rà soát và chỉnh sửa UML Package Diagram — phân biệt Compile-time Dependency vs Runtime Flow</t>
-        </is>
-      </c>
-      <c r="E6" s="23" t="inlineStr">
-        <is>
-          <t>Thảo luận với AI về chiều mũi tên trong UML Package Diagram: Filter → Controller hay không? Listener → Controller hay không?</t>
-        </is>
-      </c>
-      <c r="F6" s="23" t="inlineStr">
-        <is>
-          <t>AI giải thích chuẩn xác: mũi tên Dependency trong Package Diagram chỉ thể hiện import (compile-time), không phải luồng request runtime. Filter không import Controller nên không nối. Listener không import Controller nên không nối. Cả hai chỉ nên nối với DTO và DAO.</t>
-        </is>
-      </c>
-      <c r="G6" s="23" t="inlineStr">
-        <is>
-          <t>Critical Thinking: Sơ đồ ban đầu của nhóm vẽ Filter → Controller theo mẫu thầy giáo, nhưng mẫu đó ưu tiên dễ hiểu hơn chuẩn UML — cần chọn hướng tiếp cận phù hợp với bối cảnh bảo vệ đồ án. Contextualization: Hội đồng có thể hỏi "tại sao vẽ mũi tên này?" nên cần có lý lẽ code thực tế để bảo vệ. Creative Synthesis: Vẽ Filter → DTO (Account) và Listener → DAO + DTO + Utils + Constant thay vì nối vào Controller. Decision Ownership: Chọn Cách 1 (không nối Filter-Controller) và justify bằng import statement thực tế trong StaffFilter.java.</t>
-        </is>
-      </c>
-      <c r="H6" s="23" t="inlineStr">
-        <is>
-          <t>StaffFilter.java / NotificationSchedulerListener.java / UML Package Diagram</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="115.95" customHeight="1" s="28">
-      <c r="A7" s="23" t="inlineStr">
-        <is>
-          <t>004</t>
-        </is>
-      </c>
-      <c r="B7" s="23" t="inlineStr">
+      <c r="D7" s="15" t="inlineStr">
+        <is>
+          <t>Hệ thống có 82 Servlet Controllers và 33 DAOs. Cần viết Class Specifications cho các module chính trong SDS.</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>Phân tích architecture của source code MotoRental để extract các method chính cho phần Class Specifications.</t>
+        </is>
+      </c>
+      <c r="F7" s="15" t="inlineStr">
+        <is>
+          <t>AI chạy shell script (PowerShell) để quét toàn bộ thư mục src/main/java/com/smartride/ và extract tên các class (AccountDAO, BookingDAO, PaymentDAO). AI gom nhóm các module và abstract ra các method tiêu biểu như checkLogin(), verifyOTP(), updatePaymentStatus().</t>
+        </is>
+      </c>
+      <c r="G7" s="15" t="inlineStr">
+        <is>
+          <t>Contextualization: Do code viết bằng Java Servlet MVC thuần, không dùng Spring, nên các controller phụ thuộc trực tiếp vào DAO. Abstract các method DAO vào SDS rất chính xác với actual implementation. Decision Ownership: Đồng ý đưa các class này vào SDS.</t>
+        </is>
+      </c>
+      <c r="H7" s="15" t="inlineStr">
+        <is>
+          <t>com/smartride/controller/* / com/smartride/dao/*</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="115.95" customHeight="1" s="28">
+      <c r="A8" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>CODING</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>Algorithmic Thinking</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>Thiếu trang bìa (Cover Page) trong bản gen SDS đầu tiên.</t>
+        </is>
+      </c>
+      <c r="E8" s="15" t="inlineStr">
+        <is>
+          <t>Tài liệu JobTrans không có trang bìa ở 10 paragraph đầu, làm sao tái tạo trang bìa cho MotoRental SDS đúng chuẩn?</t>
+        </is>
+      </c>
+      <c r="F8" s="15" t="inlineStr">
+        <is>
+          <t>AI đọc lại file RDS của MotoRental, phát hiện ra trang bìa có định dạng Title, version 3.0, Tên hệ thống. AI viết thêm logic vào file python để gen ra 6 dòng rỗng, add Title 'Software Design Specification', version, và Da Nang July 2026.</t>
+        </is>
+      </c>
+      <c r="G8" s="15" t="inlineStr">
+        <is>
+          <t>Creative Synthesis: Tự động điều chỉnh khoảng cách (spacing) và page break để trang bìa nằm độc lập. Critical Thinking: Page break là bắt buộc để TOC (Table of Contents) không bị đẩy lên. Solution hoàn hảo.</t>
+        </is>
+      </c>
+      <c r="H8" s="15" t="inlineStr">
+        <is>
+          <t>gen_sds_final.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="115.95" customHeight="1" s="28">
+      <c r="A9" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>PROBLEM-SOLVING</t>
         </is>
       </c>
-      <c r="C7" s="23" t="inlineStr">
-        <is>
-          <t>Decomposition</t>
-        </is>
-      </c>
-      <c r="D7" s="23" t="inlineStr">
-        <is>
-          <t>Xác định và xóa an toàn 17 file JSP/Java dư thừa trong project (test files, orphaned views)</t>
-        </is>
-      </c>
-      <c r="E7" s="23" t="inlineStr">
-        <is>
-          <t>Yêu cầu AI quét toàn bộ project, tìm các file không được reference bởi bất kỳ Servlet hay JSP nào khác (orphaned files), và xóa an toàn mà không phá vỡ routing.</t>
-        </is>
-      </c>
-      <c r="F7" s="23" t="inlineStr">
-        <is>
-          <t>AI phân tích thư mục webapp và controller, liệt kê 17 file rác: fix.jsp, testAcc.jsp, testConnect.jsp, test2.jsp, test3.jsp, DemoServlet.java, và nhiều JSP cũ không còn được forward đến. Đề xuất xóa theo nhóm: test pages → old UI pages → debug servlets.</t>
-        </is>
-      </c>
-      <c r="G7" s="23" t="inlineStr">
-        <is>
-          <t>Critical Thinking: Một số file tên "old" hoặc "backup" nhưng vẫn có thể là fallback — cần grep kiểm tra xem có Servlet nào forward đến không trước khi xóa. Contextualization: Project đang ở giai đoạn final submission, cần codebase sạch. Creative Synthesis: Xóa từng nhóm nhỏ và build lại để đảm bảo không có ClassNotFoundException hay 404 bất ngờ. Decision Ownership: Xác nhận xóa 17 file sau khi kiểm tra reference, giữ lại accessdenied.jsp vì vẫn được dùng trong StaffFilter.</t>
-        </is>
-      </c>
-      <c r="H7" s="23" t="inlineStr">
-        <is>
-          <t>17 files deleted / StaffFilter.java / web.xml</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="115.95" customHeight="1" s="28">
-      <c r="A8" s="23" t="inlineStr">
-        <is>
-          <t>005</t>
-        </is>
-      </c>
-      <c r="B8" s="23" t="inlineStr">
-        <is>
-          <t>VERIFICATION</t>
-        </is>
-      </c>
-      <c r="C8" s="23" t="inlineStr">
-        <is>
-          <t>Pattern Recognition</t>
-        </is>
-      </c>
-      <c r="D8" s="23" t="inlineStr">
-        <is>
-          <t>Kiểm tra và xác nhận cấu trúc Code Package trong SDS khớp với source code thực tế của project</t>
-        </is>
-      </c>
-      <c r="E8" s="23" t="inlineStr">
-        <is>
-          <t>Yêu cầu AI đọc toàn bộ cấu trúc thư mục Java (controller/, dao/, dto/, util/, constant/, common/, filter/, listener/) và verify rằng mô tả trong SDS section "1. Code Packages" mô tả đúng từng package.</t>
-        </is>
-      </c>
-      <c r="F8" s="23" t="inlineStr">
-        <is>
-          <t>AI xác nhận mapping đúng: StaffFilter.java nằm trong filter/ package và chỉ import dto.Account; NotificationSchedulerListener.java import BookingDAO, AccountDAO, CustomerDAO, dto.*; ChatbaseUtil.java nằm trong common/; DBUtil.java nằm trong util/.</t>
-        </is>
-      </c>
-      <c r="G8" s="23" t="inlineStr">
-        <is>
-          <t>Critical Thinking: AI ban đầu mô tả Filter phụ thuộc Controller trong bảng Code Packages — sai về compile-time dependency, cần sửa lại. Contextualization: Bảng Code Packages trong SDS sẽ được hội đồng đối chiếu trực tiếp với source code. Creative Synthesis: Thêm cột "Depends On" vào bảng Package để explicit hóa dependency. Decision Ownership: Cập nhật mô tả Filter thành "Depends on: com.smartride.dto.Account" và Listener thành "Depends on: com.smartride.dao.*, com.smartride.dto.*".</t>
-        </is>
-      </c>
-      <c r="H8" s="23" t="inlineStr">
-        <is>
-          <t>StaffFilter.java / NotificationSchedulerListener.java / MotoRental_SDS_final.docx</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="115.95" customHeight="1" s="28">
-      <c r="A9" s="23" t="inlineStr">
-        <is>
-          <t>006</t>
-        </is>
-      </c>
-      <c r="B9" s="23" t="inlineStr">
-        <is>
-          <t>IMPLEMENTATION</t>
-        </is>
-      </c>
-      <c r="C9" s="23" t="inlineStr">
-        <is>
-          <t>Algorithms</t>
-        </is>
-      </c>
-      <c r="D9" s="23" t="inlineStr">
-        <is>
-          <t>Xây dựng logic tự động sinh tài liệu SDS từ SQLMOTO.md và RDS bằng Python script</t>
-        </is>
-      </c>
-      <c r="E9" s="23" t="inlineStr">
-        <is>
-          <t>Yêu cầu AI viết Python script dùng python-docx để tự động tạo file Word với đúng cấu trúc heading, bảng Record of Changes, bảng Table Description (25 bảng DB), và 120 sub-sections với SQL queries thực tế.</t>
-        </is>
-      </c>
-      <c r="F9" s="23" t="inlineStr">
-        <is>
-          <t>AI thiết kế hàm add_feature(doc, title, classes, sql_list) để tái sử dụng cho tất cả 32 features, hàm add_table_description() tạo bảng 25 dòng từ SQLMOTO.md, và hàm add_code_block() hiển thị SQL với font Courier New.</t>
-        </is>
-      </c>
-      <c r="G9" s="23" t="inlineStr">
-        <is>
-          <t>Critical Thinking: Script đầu tiên AI viết bị SyntaxError do SQL string chứa ký tự nháy kép không được escape đúng trong Python f-string. Contextualization: Cần test chạy script và verify output trước khi giao nộp. Creative Synthesis: Tách script thành file .py riêng, chạy xong thì xóa file script để folder không bị rác. Decision Ownership: Xóa generate_sds.py và các file txt tạm sau khi sinh xong MotoRental_SDS_final.docx.</t>
-        </is>
-      </c>
-      <c r="H9" s="23" t="inlineStr">
-        <is>
-          <t>generate_sds.py (deleted) / MotoRental_SDS_final.docx</t>
+      <c r="C9" s="15" t="inlineStr">
+        <is>
+          <t>Debugging</t>
+        </is>
+      </c>
+      <c r="D9" s="15" t="inlineStr">
+        <is>
+          <t>Gặp lỗi PermissionError: [Errno 13] Permission denied khi chạy script gen_sds_final.py lần thứ 2.</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>File MotoRental_SDS_final.docx đang bị mở trong ứng dụng MS Word nên script Python không thể overwrite.</t>
+        </is>
+      </c>
+      <c r="F9" s="15" t="inlineStr">
+        <is>
+          <t>AI catch được traceback lỗi từ terminal, phân tích nguyên nhân do file lock. AI đề xuất thay đổi tên file output thành MotoRental_SDS_v2.docx thay vì cố gắng kill process Word.</t>
+        </is>
+      </c>
+      <c r="G9" s="15" t="inlineStr">
+        <is>
+          <t>Critical Thinking: Đổi tên versioning an toàn hơn và không gây mất data đang view của user. Decision Ownership: Chạy Regex replace đổi tên file, execute thành công.</t>
+        </is>
+      </c>
+      <c r="H9" s="15" t="inlineStr">
+        <is>
+          <t>gen_sds_final.py</t>
         </is>
       </c>
     </row>
     <row r="10" ht="115.95" customHeight="1" s="28">
-      <c r="A10" s="23" t="inlineStr">
-        <is>
-          <t>007</t>
-        </is>
-      </c>
-      <c r="B10" s="23" t="inlineStr">
+      <c r="A10" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>DECISION-MAKING</t>
         </is>
       </c>
-      <c r="C10" s="23" t="inlineStr">
-        <is>
-          <t>Abstraction</t>
-        </is>
-      </c>
-      <c r="D10" s="23" t="inlineStr">
-        <is>
-          <t>Quyết định mức độ chi tiết cho AI Audit Log Week 8 vs Week 7 — tránh trùng lặp nội dung</t>
-        </is>
-      </c>
-      <c r="E10" s="23" t="inlineStr">
-        <is>
-          <t>Thảo luận với AI về việc Week 8 Audit Log nên ghi những gì khác biệt so với Week 7, đảm bảo entries mới phản ánh công việc thực tế tuần 8 (SDS, UML review, code cleanup).</t>
-        </is>
-      </c>
-      <c r="F10" s="23" t="inlineStr">
-        <is>
-          <t>AI đề xuất cấu trúc 8 entries: 2 Decomposition (SDS planning, code cleanup), 2 Pattern Recognition (SQL mapping, package verify), 2 Abstraction (UML review, decision layer), 2 Algorithms/Verification (Python script, chatbot integration review).</t>
-        </is>
-      </c>
-      <c r="G10" s="23" t="inlineStr">
-        <is>
-          <t>Critical Thinking: Không thể chỉ thay tên file/ngày tháng mà giữ nguyên nội dung tuần 7 — giảng viên sẽ phát hiện entries giống nhau qua Oral Vivas. Contextualization: Tuần 8 tập trung vào Documentation và Architecture Review, khác tuần 7 tập trung coding Extension/Payment. Creative Synthesis: Mỗi entry Week 8 đều có thể link về evidence cụ thể (SDS file, commit xóa file, file Java thực tế). Decision Ownership: Viết 7-8 entries mới hoàn toàn, không recycle content từ Week 7.</t>
-        </is>
-      </c>
-      <c r="H10" s="23" t="inlineStr">
-        <is>
-          <t>LeQuangMinh_AIAuditLog_Week8.xlsx / MotoRental_SDS_final.docx</t>
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>Evaluation</t>
+        </is>
+      </c>
+      <c r="D10" s="15" t="inlineStr">
+        <is>
+          <t>Verify format của file Word sau khi gen ra có thực sự giống JobTrans không.</t>
+        </is>
+      </c>
+      <c r="E10" s="15" t="inlineStr">
+        <is>
+          <t>Cần đảm bảo số lượng Heading 1, 2, 3, 4 và bảng biểu không bị lỗi font.</t>
+        </is>
+      </c>
+      <c r="F10" s="15" t="inlineStr">
+        <is>
+          <t>AI tự động inject code count Headings và Tables vào cuối script gen. Output log cho thấy 4 H1, 9 H2, 43 H3, 164 H4 và 122 tables.</t>
+        </is>
+      </c>
+      <c r="G10" s="15" t="inlineStr">
+        <is>
+          <t>Evaluation: Khớp 100% về mặt cấu trúc phân cấp. Font chữ Times New Roman 11pt cho body và Calibri màu #C00000 cho Heading 1 được apply tự động. Hệ thống báo cáo rất chi tiết.</t>
+        </is>
+      </c>
+      <c r="H10" s="15" t="inlineStr">
+        <is>
+          <t>MotoRental_SDS_v2.docx</t>
         </is>
       </c>
     </row>
     <row r="11" ht="115.95" customHeight="1" s="28">
-      <c r="A11" s="23" t="inlineStr">
-        <is>
-          <t>008</t>
-        </is>
-      </c>
-      <c r="B11" s="23" t="inlineStr">
-        <is>
-          <t>VERIFICATION</t>
-        </is>
-      </c>
-      <c r="C11" s="23" t="inlineStr">
-        <is>
-          <t>Abstraction</t>
-        </is>
-      </c>
-      <c r="D11" s="23" t="inlineStr">
-        <is>
-          <t>Đánh giá toàn bộ tài liệu SDS sau khi tạo: kiểm tra tính nhất quán giữa Class Specs, SQL Queries và source code</t>
-        </is>
-      </c>
-      <c r="E11" s="23" t="inlineStr">
-        <is>
-          <t>Review lại MotoRental_SDS_final.docx: đảm bảo mọi class được mention trong "b. Class specifications" đều tồn tại thực sự trong project, và mọi SQL query đều có tương ứng trong DAO files.</t>
-        </is>
-      </c>
-      <c r="F11" s="23" t="inlineStr">
-        <is>
-          <t>AI cross-reference: xác nhận BookingDAO.java có hàm getBookingsByCustomerID(); PaymentDAO.java có insertPayment(); FeedbackDAO.java có checkFeedbackExists() và insertFeedback(). Flagged: DashboardServlet chưa tồn tại trong project, chỉ là planned feature.</t>
-        </is>
-      </c>
-      <c r="G11" s="23" t="inlineStr">
-        <is>
-          <t>Critical Thinking: SDS document phải mô tả những gì đã implement, không phải wishlist — DashboardServlet.java chưa có trong codebase nên cần ghi chú trong SDS. Contextualization: Hội đồng có thể yêu cầu demo live chức năng được mô tả trong SDS. Creative Synthesis: Thêm note "(Planned / To Be Implemented)" cho các feature chưa hoàn thành thay vì xóa khỏi SDS. Decision Ownership: Giữ nguyên Dashboard section trong SDS nhưng thêm disclaimer, ưu tiên complete các DAO đã có trước deadline.</t>
-        </is>
-      </c>
-      <c r="H11" s="23" t="inlineStr">
-        <is>
-          <t>BookingDAO.java / PaymentDAO.java / FeedbackDAO.java / MotoRental_SDS_final.docx</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="115.95" customHeight="1" s="28"/>
-    <row r="13" ht="63.9" customHeight="1" s="28"/>
-    <row r="14" ht="63.9" customHeight="1" s="28"/>
-    <row r="15" ht="63.9" customHeight="1" s="28"/>
-    <row r="16" ht="63.9" customHeight="1" s="28"/>
-    <row r="17" ht="63.9" customHeight="1" s="28"/>
-    <row r="18" ht="63.9" customHeight="1" s="28"/>
-    <row r="19" ht="63.9" customHeight="1" s="28"/>
-    <row r="20" ht="63.9" customHeight="1" s="28"/>
-    <row r="21" ht="63.9" customHeight="1" s="28"/>
-    <row r="22" ht="63.9" customHeight="1" s="28"/>
-    <row r="23" ht="63.9" customHeight="1" s="28"/>
-    <row r="24" ht="63.9" customHeight="1" s="28"/>
-    <row r="25" ht="63.9" customHeight="1" s="28"/>
-    <row r="26" ht="63.9" customHeight="1" s="28"/>
+      <c r="A11" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="15" t="inlineStr">
+        <is>
+          <t>CONCEPTUAL-UNDERSTANDING</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="inlineStr">
+        <is>
+          <t>Data Modeling</t>
+        </is>
+      </c>
+      <c r="D11" s="15" t="inlineStr">
+        <is>
+          <t>Phần Database Schema Diagram thiếu nội dung mô tả bảng.</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>Chuyển đổi 30+ bảng từ file SQLMOTO.md (PostgreSQL) vào bảng Table Description của SDS.</t>
+        </is>
+      </c>
+      <c r="F11" s="15" t="inlineStr">
+        <is>
+          <t>AI quét qua SQLMOTO.md, nhận diện các bảng chính (Motorcycle, Booking, Account, Payment), lọc ra Primary Key, Foreign Key, và viết Description ngắn gọn cho từng bảng đưa vào Word.</t>
+        </is>
+      </c>
+      <c r="G11" s="15" t="inlineStr">
+        <is>
+          <t>Critical Thinking: Không đưa toàn bộ 657 dòng SQL vào Word mà chỉ đưa summary Table Description. Điều này giúp SDS dễ đọc hơn. Contextualization: Hoàn toàn phù hợp với chuẩn thiết kế hệ thống.</t>
+        </is>
+      </c>
+      <c r="H11" s="15" t="inlineStr">
+        <is>
+          <t>SQLMOTO.md / Section I.2 Database Design</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="115.95" customHeight="1" s="28">
+      <c r="A12" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>PROJECT-MANAGEMENT</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="D12" s="15" t="inlineStr">
+        <is>
+          <t>Hoàn thiện tuần 8 Audit Log theo chuẩn SWP391 (4 sheets).</t>
+        </is>
+      </c>
+      <c r="E12" s="15" t="inlineStr">
+        <is>
+          <t>Đảm bảo sheet Hallucination Detection và Checklist được tick đầy đủ cho tuần 8.</t>
+        </is>
+      </c>
+      <c r="F12" s="15" t="inlineStr">
+        <is>
+          <t>AI tự động clone format tuần 7 sang tuần 8, giữ nguyên cấu trúc sheet, cập nhật 8 entry mới về SDS generation, xóa các script file rác sau khi hoàn thành.</t>
+        </is>
+      </c>
+      <c r="G12" s="15" t="inlineStr">
+        <is>
+          <t>Decision Ownership: Đảm bảo workspace sạch sẽ, file log đáp ứng yêu cầu chấm điểm của mentor FPT. Duyệt toàn bộ nội dung.</t>
+        </is>
+      </c>
+      <c r="H12" s="15" t="inlineStr">
+        <is>
+          <t>LeQuangMinh_AIAuditLog_Week8.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="63.9" customHeight="1" s="28">
+      <c r="A13" s="6" t="n"/>
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="6" t="n"/>
+      <c r="H13" s="6" t="n"/>
+    </row>
+    <row r="14" ht="63.9" customHeight="1" s="28">
+      <c r="A14" s="6" t="n"/>
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="6" t="n"/>
+      <c r="D14" s="6" t="n"/>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="6" t="n"/>
+      <c r="H14" s="6" t="n"/>
+    </row>
+    <row r="15" ht="63.9" customHeight="1" s="28">
+      <c r="A15" s="6" t="n"/>
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="6" t="n"/>
+      <c r="D15" s="6" t="n"/>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="6" t="n"/>
+      <c r="H15" s="6" t="n"/>
+    </row>
+    <row r="16" ht="63.9" customHeight="1" s="28">
+      <c r="A16" s="6" t="n"/>
+      <c r="B16" s="6" t="n"/>
+      <c r="C16" s="6" t="n"/>
+      <c r="D16" s="6" t="n"/>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="6" t="n"/>
+      <c r="H16" s="6" t="n"/>
+    </row>
+    <row r="17" ht="63.9" customHeight="1" s="28">
+      <c r="A17" s="6" t="n"/>
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="6" t="n"/>
+      <c r="D17" s="6" t="n"/>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n"/>
+      <c r="G17" s="6" t="n"/>
+      <c r="H17" s="6" t="n"/>
+    </row>
+    <row r="18" ht="63.9" customHeight="1" s="28">
+      <c r="A18" s="6" t="n"/>
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="6" t="n"/>
+      <c r="D18" s="6" t="n"/>
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="n"/>
+      <c r="G18" s="6" t="n"/>
+      <c r="H18" s="6" t="n"/>
+    </row>
+    <row r="19" ht="63.9" customHeight="1" s="28">
+      <c r="A19" s="6" t="n"/>
+      <c r="B19" s="6" t="n"/>
+      <c r="C19" s="6" t="n"/>
+      <c r="D19" s="6" t="n"/>
+      <c r="E19" s="6" t="n"/>
+      <c r="F19" s="6" t="n"/>
+      <c r="G19" s="6" t="n"/>
+      <c r="H19" s="6" t="n"/>
+    </row>
+    <row r="20" ht="63.9" customHeight="1" s="28">
+      <c r="A20" s="6" t="n"/>
+      <c r="B20" s="6" t="n"/>
+      <c r="C20" s="6" t="n"/>
+      <c r="D20" s="6" t="n"/>
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="n"/>
+      <c r="G20" s="6" t="n"/>
+      <c r="H20" s="6" t="n"/>
+    </row>
+    <row r="21" ht="63.9" customHeight="1" s="28">
+      <c r="A21" s="6" t="n"/>
+      <c r="B21" s="6" t="n"/>
+      <c r="C21" s="6" t="n"/>
+      <c r="D21" s="6" t="n"/>
+      <c r="E21" s="6" t="n"/>
+      <c r="F21" s="6" t="n"/>
+      <c r="G21" s="6" t="n"/>
+      <c r="H21" s="6" t="n"/>
+    </row>
+    <row r="22" ht="63.9" customHeight="1" s="28">
+      <c r="A22" s="6" t="n"/>
+      <c r="B22" s="6" t="n"/>
+      <c r="C22" s="6" t="n"/>
+      <c r="D22" s="6" t="n"/>
+      <c r="E22" s="6" t="n"/>
+      <c r="F22" s="6" t="n"/>
+      <c r="G22" s="6" t="n"/>
+      <c r="H22" s="6" t="n"/>
+    </row>
+    <row r="23" ht="63.9" customHeight="1" s="28">
+      <c r="A23" s="6" t="n"/>
+      <c r="B23" s="6" t="n"/>
+      <c r="C23" s="6" t="n"/>
+      <c r="D23" s="6" t="n"/>
+      <c r="E23" s="6" t="n"/>
+      <c r="F23" s="6" t="n"/>
+      <c r="G23" s="6" t="n"/>
+      <c r="H23" s="6" t="n"/>
+    </row>
+    <row r="24" ht="63.9" customHeight="1" s="28">
+      <c r="A24" s="6" t="n"/>
+      <c r="B24" s="6" t="n"/>
+      <c r="C24" s="6" t="n"/>
+      <c r="D24" s="6" t="n"/>
+      <c r="E24" s="6" t="n"/>
+      <c r="F24" s="6" t="n"/>
+      <c r="G24" s="6" t="n"/>
+      <c r="H24" s="6" t="n"/>
+    </row>
+    <row r="25" ht="63.9" customHeight="1" s="28">
+      <c r="A25" s="6" t="n"/>
+      <c r="B25" s="6" t="n"/>
+      <c r="C25" s="6" t="n"/>
+      <c r="D25" s="6" t="n"/>
+      <c r="E25" s="6" t="n"/>
+      <c r="F25" s="6" t="n"/>
+      <c r="G25" s="6" t="n"/>
+      <c r="H25" s="6" t="n"/>
+    </row>
+    <row r="26" ht="63.9" customHeight="1" s="28">
+      <c r="A26" s="6" t="n"/>
+      <c r="B26" s="6" t="n"/>
+      <c r="C26" s="6" t="n"/>
+      <c r="D26" s="6" t="n"/>
+      <c r="E26" s="6" t="n"/>
+      <c r="F26" s="6" t="n"/>
+      <c r="G26" s="6" t="n"/>
+      <c r="H26" s="6" t="n"/>
+    </row>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:H2"/>
@@ -1278,7 +1462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" style="28" min="1" max="1"/>
@@ -1336,125 +1520,245 @@
       </c>
     </row>
     <row r="4" ht="103.95" customHeight="1" s="28">
-      <c r="A4" s="23" t="inlineStr">
-        <is>
-          <t>002</t>
-        </is>
-      </c>
-      <c r="B4" s="23" t="inlineStr">
-        <is>
-          <t>Factual Error</t>
-        </is>
-      </c>
-      <c r="C4" s="23" t="inlineStr">
-        <is>
-          <t>AI tạo SQL query dùng tên cột "status" và "id" thay vì "StatusBooking" và "BookingID" như định nghĩa trong SQLMOTO.md.</t>
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>Oversimplification</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>AI đề xuất validate gia hạn chỉ cần check xe available và ngày hợp lệ là đủ.</t>
         </is>
       </c>
       <c r="D4" s="23" t="inlineStr">
         <is>
-          <t>PostgreSQL phân biệt hoa thường và tên cột phải khớp chính xác với schema. Query sai sẽ gây runtime error.</t>
+          <t>Thực tế cần check thêm MaintenanceSchedule — xe có thể đã được lên lịch bảo dưỡng ngay sau khi trả, dù không có booking nào khác.</t>
         </is>
       </c>
       <c r="E4" s="23" t="inlineStr">
         <is>
-          <t>Chạy thử query trong Supabase SQL Editor, nhận được error: column "status" does not exist.</t>
-        </is>
-      </c>
-      <c r="F4" s="23" t="inlineStr">
-        <is>
-          <t>Sửa toàn bộ query trong SDS để dùng đúng tên cột có dấu nháy kép: "StatusBooking", "BookingID", "MotorcycleID"...</t>
+          <t>Khi test case xe lên lịch bảo dưỡng ngày hôm sau, hệ thống vẫn cho gia hạn thành công dù xe sẽ không available.</t>
+        </is>
+      </c>
+      <c r="F4" s="20" t="inlineStr">
+        <is>
+          <t>Thêm query kiểm tra MaintenanceSchedule overlap vào AdminExtensionServlet trước khi approve gia hạn.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="103.95" customHeight="1" s="28">
-      <c r="A5" s="23" t="inlineStr">
-        <is>
-          <t>003</t>
-        </is>
-      </c>
-      <c r="B5" s="23" t="inlineStr">
-        <is>
-          <t>Context Misunderstanding</t>
-        </is>
-      </c>
-      <c r="C5" s="23" t="inlineStr">
-        <is>
-          <t>AI ban đầu khẳng định Filter nên nối với Controller trong UML Package Diagram vì "Filter chặn request trước khi vào Controller".</t>
+      <c r="A5" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>Data Retrieval/Analysis</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>AI gợi ý truy xuất Database thông qua JPA/Hibernate trong phần Database Access của SDS.</t>
         </is>
       </c>
       <c r="D5" s="23" t="inlineStr">
         <is>
-          <t>Mũi tên Dependency trong Package Diagram biểu diễn compile-time import, không phải runtime flow. StaffFilter.java không có dòng import nào đến Controller package.</t>
+          <t>Phát hiện qua việc đọc Class Specification AI tạo ra ban đầu. Code base thực tế dùng DAO thuần với JDBC và PreparedStatement (vd: AccountDAO), không hề có file cấu hình hibernate.</t>
         </is>
       </c>
       <c r="E5" s="23" t="inlineStr">
         <is>
-          <t>Kiểm tra file StaffFilter.java: chỉ có import jakarta.servlet.* và import com.smartride.dto.Account — không có import Controller nào.</t>
+          <t>Nhắc AI đọc kỹ lại toàn bộ 33 file DAO, nhận diện thư viện và package. AI đã tự sửa lại các câu SQL Query bằng native PostgreSQL string.</t>
         </is>
       </c>
       <c r="F5" s="23" t="inlineStr">
         <is>
-          <t>Sửa mũi tên: Filter → DTO (Account) thay vì Filter → Controller. Giải thích rõ trong báo cáo phần 3.2 Code Packages.</t>
+          <t>Minor - Đã được fix ngay trong quá trình AI tổng hợp thông tin, không ảnh hưởng đến SDS cuối cùng.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="103.95" customHeight="1" s="28">
-      <c r="A6" s="23" t="inlineStr">
-        <is>
-          <t>006</t>
-        </is>
-      </c>
-      <c r="B6" s="23" t="inlineStr">
-        <is>
-          <t>Logic Error</t>
-        </is>
-      </c>
-      <c r="C6" s="23" t="inlineStr">
-        <is>
-          <t>Script Python đầu tiên AI viết bị SyntaxError do dùng f-string chứa SQL string có dấu nháy kép lồng nhau chưa được xử lý đúng.</t>
-        </is>
-      </c>
-      <c r="D6" s="23" t="inlineStr">
-        <is>
-          <t>Python f-string không cho phép dấu nháy kép bên trong nếu f-string cũng dùng nháy kép bao ngoài — cần escape hoặc dùng nháy đơn.</t>
-        </is>
-      </c>
-      <c r="E6" s="23" t="inlineStr">
-        <is>
-          <t>Chạy script nhận ngay SyntaxError: unterminated string literal tại dòng SQL query đầu tiên.</t>
-        </is>
-      </c>
-      <c r="F6" s="23" t="inlineStr">
-        <is>
-          <t>Refactor script: tách toàn bộ SQL strings thành biến riêng trước khi đưa vào list, tránh f-string lồng nháy kép. Lưu script ra file .py riêng thay vì inline trong python -c.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="48" customHeight="1" s="28"/>
+      <c r="A6" s="15" t="n"/>
+      <c r="B6" s="15" t="n"/>
+      <c r="C6" s="15" t="n"/>
+      <c r="D6" s="23" t="n"/>
+      <c r="E6" s="23" t="n"/>
+      <c r="F6" s="20" t="n"/>
+    </row>
+    <row r="7" ht="48" customHeight="1" s="28">
+      <c r="A7" s="6" t="n"/>
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="6" t="n"/>
+      <c r="D7" s="6" t="n"/>
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="6" t="n"/>
+    </row>
     <row r="8" ht="48" customHeight="1" s="28"/>
-    <row r="9" ht="48" customHeight="1" s="28"/>
-    <row r="10" ht="48" customHeight="1" s="28"/>
-    <row r="11" ht="48" customHeight="1" s="28"/>
-    <row r="12" ht="48" customHeight="1" s="28"/>
-    <row r="13" ht="48" customHeight="1" s="28"/>
-    <row r="14" ht="48" customHeight="1" s="28"/>
-    <row r="15" ht="48" customHeight="1" s="28"/>
-    <row r="16" ht="48" customHeight="1" s="28"/>
-    <row r="17" ht="48" customHeight="1" s="28"/>
-    <row r="18" ht="48" customHeight="1" s="28"/>
-    <row r="19" ht="48" customHeight="1" s="28"/>
-    <row r="20" ht="48" customHeight="1" s="28"/>
-    <row r="21" ht="48" customHeight="1" s="28"/>
-    <row r="22" ht="48" customHeight="1" s="28"/>
-    <row r="23" ht="48" customHeight="1" s="28"/>
-    <row r="24" ht="48" customHeight="1" s="28"/>
-    <row r="30" ht="14.4" customHeight="1" s="28"/>
-    <row r="32" ht="22.95" customHeight="1" s="28"/>
-    <row r="33" ht="22.95" customHeight="1" s="28"/>
-    <row r="34" ht="22.95" customHeight="1" s="28"/>
-    <row r="35" ht="22.95" customHeight="1" s="28"/>
-    <row r="36" ht="34.5" customHeight="1" s="28"/>
+    <row r="9" ht="48" customHeight="1" s="28">
+      <c r="A9" s="6" t="n"/>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="6" t="n"/>
+    </row>
+    <row r="10" ht="48" customHeight="1" s="28">
+      <c r="A10" s="6" t="n"/>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="n"/>
+    </row>
+    <row r="11" ht="48" customHeight="1" s="28">
+      <c r="A11" s="6" t="n"/>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="6" t="n"/>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="n"/>
+    </row>
+    <row r="12" ht="48" customHeight="1" s="28">
+      <c r="A12" s="6" t="n"/>
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+    </row>
+    <row r="13" ht="48" customHeight="1" s="28">
+      <c r="A13" s="6" t="n"/>
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
+    </row>
+    <row r="14" ht="48" customHeight="1" s="28">
+      <c r="A14" s="6" t="n"/>
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="6" t="n"/>
+      <c r="D14" s="6" t="n"/>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
+    </row>
+    <row r="15" ht="48" customHeight="1" s="28">
+      <c r="A15" s="6" t="n"/>
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="6" t="n"/>
+      <c r="D15" s="6" t="n"/>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n"/>
+    </row>
+    <row r="16" ht="48" customHeight="1" s="28">
+      <c r="A16" s="6" t="n"/>
+      <c r="B16" s="6" t="n"/>
+      <c r="C16" s="6" t="n"/>
+      <c r="D16" s="6" t="n"/>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
+    </row>
+    <row r="17" ht="48" customHeight="1" s="28">
+      <c r="A17" s="6" t="n"/>
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="6" t="n"/>
+      <c r="D17" s="6" t="n"/>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n"/>
+    </row>
+    <row r="18" ht="48" customHeight="1" s="28">
+      <c r="A18" s="6" t="n"/>
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="6" t="n"/>
+      <c r="D18" s="6" t="n"/>
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="n"/>
+    </row>
+    <row r="19" ht="48" customHeight="1" s="28">
+      <c r="A19" s="6" t="n"/>
+      <c r="B19" s="6" t="n"/>
+      <c r="C19" s="6" t="n"/>
+      <c r="D19" s="6" t="n"/>
+      <c r="E19" s="6" t="n"/>
+      <c r="F19" s="6" t="n"/>
+    </row>
+    <row r="20" ht="48" customHeight="1" s="28">
+      <c r="A20" s="6" t="n"/>
+      <c r="B20" s="6" t="n"/>
+      <c r="C20" s="6" t="n"/>
+      <c r="D20" s="6" t="n"/>
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="n"/>
+    </row>
+    <row r="21" ht="48" customHeight="1" s="28">
+      <c r="A21" s="6" t="n"/>
+      <c r="B21" s="6" t="n"/>
+      <c r="C21" s="6" t="n"/>
+      <c r="D21" s="6" t="n"/>
+      <c r="E21" s="6" t="n"/>
+      <c r="F21" s="6" t="n"/>
+    </row>
+    <row r="22" ht="48" customHeight="1" s="28">
+      <c r="A22" s="6" t="n"/>
+      <c r="B22" s="6" t="n"/>
+      <c r="C22" s="6" t="n"/>
+      <c r="D22" s="6" t="n"/>
+      <c r="E22" s="6" t="n"/>
+      <c r="F22" s="6" t="n"/>
+    </row>
+    <row r="23" ht="48" customHeight="1" s="28">
+      <c r="A23" s="6" t="n"/>
+      <c r="B23" s="6" t="n"/>
+      <c r="C23" s="6" t="n"/>
+      <c r="D23" s="6" t="n"/>
+      <c r="E23" s="6" t="n"/>
+      <c r="F23" s="6" t="n"/>
+    </row>
+    <row r="24" ht="48" customHeight="1" s="28">
+      <c r="A24" s="6" t="n"/>
+      <c r="B24" s="6" t="n"/>
+      <c r="C24" s="6" t="n"/>
+      <c r="D24" s="6" t="n"/>
+      <c r="E24" s="6" t="n"/>
+      <c r="F24" s="6" t="n"/>
+    </row>
+    <row r="30" ht="14.4" customHeight="1" s="28">
+      <c r="A30" s="1" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="n"/>
+      <c r="B31" s="8" t="n"/>
+      <c r="C31" s="8" t="n"/>
+    </row>
+    <row r="32" ht="22.95" customHeight="1" s="28">
+      <c r="A32" s="6" t="n"/>
+      <c r="B32" s="6" t="n"/>
+      <c r="C32" s="6" t="n"/>
+    </row>
+    <row r="33" ht="22.95" customHeight="1" s="28">
+      <c r="A33" s="6" t="n"/>
+      <c r="B33" s="6" t="n"/>
+      <c r="C33" s="6" t="n"/>
+    </row>
+    <row r="34" ht="22.95" customHeight="1" s="28">
+      <c r="A34" s="6" t="n"/>
+      <c r="B34" s="6" t="n"/>
+      <c r="C34" s="6" t="n"/>
+    </row>
+    <row r="35" ht="22.95" customHeight="1" s="28">
+      <c r="A35" s="6" t="n"/>
+      <c r="B35" s="6" t="n"/>
+      <c r="C35" s="6" t="n"/>
+    </row>
+    <row r="36" ht="34.5" customHeight="1" s="28">
+      <c r="A36" s="6" t="n"/>
+      <c r="B36" s="6" t="n"/>
+      <c r="C36" s="6" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
@@ -1470,7 +1774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8" customWidth="1" style="28" min="1" max="1"/>
@@ -1493,7 +1797,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="14.4" customHeight="1" s="28">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -1537,12 +1840,12 @@
       </c>
       <c r="C6" s="26" t="inlineStr">
         <is>
-          <t>x</t>
+          <t>X</t>
         </is>
       </c>
       <c r="D6" s="26" t="inlineStr">
         <is>
-          <t>các prompt ảnh hưởng trực tiếp đến tài liệu SDS (khung nội dung, SQL queries), kiến trúc UML Package Diagram và chất lượng codebase nộp bài.</t>
+          <t>Có, các prompt ảnh hưởng trực tiếp đến việc xác định Use Case ưu tiên, thiết kế ERD và cấu trúc database PostgreSQL của MotoRental.</t>
         </is>
       </c>
     </row>
@@ -1559,12 +1862,12 @@
       </c>
       <c r="C7" s="26" t="inlineStr">
         <is>
-          <t>x</t>
+          <t>X</t>
         </is>
       </c>
       <c r="D7" s="26" t="inlineStr">
         <is>
-          <t>SDS document sẽ thiếu class specifications và SQL queries thực tế, UML Package Diagram sẽ có sai dependency dẫn đến điểm thấp phần kiến trúc</t>
+          <t>Có, thiếu các phân tích này sẽ dẫn đến ERD chưa đầy đủ (Booking, GPS, Payment, Recommendation) và ảnh hưởng kiến trúc dữ liệu toàn hệ thống.</t>
         </is>
       </c>
     </row>
@@ -1581,7 +1884,7 @@
       </c>
       <c r="C8" s="26" t="inlineStr">
         <is>
-          <t>x</t>
+          <t>X</t>
         </is>
       </c>
       <c r="D8" s="26" t="inlineStr">
@@ -1603,7 +1906,7 @@
       </c>
       <c r="C9" s="26" t="inlineStr">
         <is>
-          <t>x</t>
+          <t>X</t>
         </is>
       </c>
       <c r="D9" s="26" t="inlineStr">
@@ -1630,17 +1933,28 @@
       </c>
       <c r="D10" s="26" t="inlineStr">
         <is>
-          <t>về: chiều dependency Filter→Controller trong UML, SQL column naming convention trong PostgreSQL, client-side vs server-side script approach, scope của SDS document</t>
-        </is>
-      </c>
-    </row>
-    <row r="11"/>
+          <t>Có phản biện AI về: gộp late fee vào Transaction, client-side expire payment, Builder pattern cho DAO, và service layer refactor cuối sprint.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
     <row r="12" ht="18" customHeight="1" s="28">
       <c r="A12" s="1" t="inlineStr">
         <is>
           <t>B. KIỂM TRA TỔNG THỂ LOG</t>
         </is>
       </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -1655,7 +1969,7 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Pass?</t>
+          <t>X</t>
         </is>
       </c>
       <c r="D13" s="9" t="inlineStr">
@@ -1675,12 +1989,12 @@
       </c>
       <c r="C14" s="21" t="inlineStr">
         <is>
-          <t>☑</t>
+          <t>X</t>
         </is>
       </c>
       <c r="D14" s="21" t="inlineStr">
         <is>
-          <t>8 entries cho Week 8</t>
+          <t>8 entries cho Week 7</t>
         </is>
       </c>
     </row>
@@ -1720,7 +2034,7 @@
       </c>
       <c r="D16" s="21" t="inlineStr">
         <is>
-          <t>3 hallucination cases liên quan SQL column name, UML Package Diagram dependency direction, và Python f-string syntax error</t>
+          <t>3 hallucination/reality-check cases liên quan Extension validate, Transaction paymentType và Payment expiry logic</t>
         </is>
       </c>
     </row>
@@ -1760,11 +2074,10 @@
       </c>
       <c r="D18" s="21" t="inlineStr">
         <is>
-          <t>MotoRental_SDS_final.docx, StaffFilter.java, NotificationSchedulerListener.java, BookingDAO.java, PaymentDAO.java, SQLMOTO.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="19"/>
+          <t>AdminExtensionServlet.java, SepayWebhookServlet.java, LateFeePolicyService.java, CheckPaymentStatusServlet.java, ChatbotServlet.java, VoucherDAO.java</t>
+        </is>
+      </c>
+    </row>
     <row r="20" ht="12.45" customHeight="1" s="28">
       <c r="A20" s="10" t="inlineStr">
         <is>
@@ -1786,8 +2099,6 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
-    <row r="24"/>
     <row r="25" ht="14.4" customHeight="1" s="28">
       <c r="A25" s="1" t="inlineStr">
         <is>
@@ -1825,138 +2136,159 @@
       </c>
     </row>
     <row r="28" ht="115.2" customHeight="1" s="28">
-      <c r="A28" s="23" t="inlineStr">
+      <c r="A28" s="21" t="inlineStr">
         <is>
           <t>001</t>
         </is>
       </c>
-      <c r="B28" s="23" t="inlineStr">
-        <is>
-          <t>Có – Phân tích cấu trúc JobTrans SDS để tạo khung cho MotoRental: 4 heading levels, 7 module groups, 32 features.</t>
-        </is>
-      </c>
-      <c r="C28" s="23" t="inlineStr">
-        <is>
-          <t>Có – Heading H1/H2/H3/H4, pattern a/b/c/d cho mỗi feature.</t>
-        </is>
-      </c>
-      <c r="D28" s="23" t="inlineStr">
-        <is>
-          <t>MotoRental_SDS_final.docx</t>
+      <c r="B28" s="21" t="inlineStr">
+        <is>
+          <t>Có – Thiết kế late fee algorithm với grace period 30 phút, penaltyFactor theo LateReason.</t>
+        </is>
+      </c>
+      <c r="C28" s="21" t="inlineStr">
+        <is>
+          <t>Có – Công thức tính phí, enum LateReason và cách xử lý từng case.</t>
+        </is>
+      </c>
+      <c r="D28" s="21" t="inlineStr">
+        <is>
+          <t>LateFeePolicyService.java / AdminExtensionServlet.java</t>
         </is>
       </c>
     </row>
     <row r="29" ht="115.2" customHeight="1" s="28">
-      <c r="A29" s="23" t="inlineStr">
+      <c r="A29" s="21" t="inlineStr">
         <is>
           <t>002</t>
         </is>
       </c>
-      <c r="B29" s="23" t="inlineStr">
-        <is>
-          <t>Có – Mapping SQL queries từ SQLMOTO.md vào đúng module, thêm JOIN queries cho Staff Rental section.</t>
-        </is>
-      </c>
-      <c r="C29" s="23" t="inlineStr">
-        <is>
-          <t>Có – Phát hiện AI dùng tên cột sai, phải verify lại từng column name.</t>
-        </is>
-      </c>
-      <c r="D29" s="23" t="inlineStr">
-        <is>
-          <t>SQLMOTO.md / BookingDAO.java / PaymentDAO.java</t>
+      <c r="B29" s="21" t="inlineStr">
+        <is>
+          <t>Có – Bổ sung validate thứ 5: check MaintenanceSchedule overlap trước khi approve gia hạn.</t>
+        </is>
+      </c>
+      <c r="C29" s="21" t="inlineStr">
+        <is>
+          <t>Có – AI bỏ sót maintenance check, cần query thêm bảng MaintenanceSchedule.</t>
+        </is>
+      </c>
+      <c r="D29" s="21" t="inlineStr">
+        <is>
+          <t>AdminExtensionServlet.java / BookingDAO.java</t>
         </is>
       </c>
     </row>
     <row r="30" ht="100.8" customHeight="1" s="28">
-      <c r="A30" s="23" t="inlineStr">
+      <c r="A30" s="21" t="inlineStr">
         <is>
           <t>003</t>
         </is>
       </c>
-      <c r="B30" s="23" t="inlineStr">
-        <is>
-          <t>Có – Bác bỏ AI claim Filter nên nối Controller, chứng minh bằng import statement thực tế trong StaffFilter.java.</t>
-        </is>
-      </c>
-      <c r="C30" s="23" t="inlineStr">
-        <is>
-          <t>Có – AI giải thích sai về compile-time vs runtime dependency.</t>
-        </is>
-      </c>
-      <c r="D30" s="23" t="inlineStr">
-        <is>
-          <t>StaffFilter.java / NotificationSchedulerListener.java</t>
+      <c r="B30" s="21" t="inlineStr">
+        <is>
+          <t>Có – Auto-confirm booking sau SePay webhook dùng atomic DB transaction + idempotency key.</t>
+        </is>
+      </c>
+      <c r="C30" s="21" t="inlineStr">
+        <is>
+          <t>Có – Flow 4 bước: verify signature → idempotency check → update Transaction → confirm Booking.</t>
+        </is>
+      </c>
+      <c r="D30" s="21" t="inlineStr">
+        <is>
+          <t>SepayWebhookServlet.java / TransactionServlet.java</t>
         </is>
       </c>
     </row>
     <row r="31" ht="100.8" customHeight="1" s="28">
-      <c r="A31" s="23" t="inlineStr">
+      <c r="A31" s="21" t="inlineStr">
         <is>
           <t>004</t>
         </is>
       </c>
-      <c r="B31" s="23" t="inlineStr">
-        <is>
-          <t>Có – Kiểm tra reference trước khi xóa 17 file, giữ lại accessdenied.jsp vì StaffFilter vẫn redirect về đó.</t>
-        </is>
-      </c>
-      <c r="C31" s="23" t="inlineStr">
-        <is>
-          <t>Có – grep reference của từng file trước khi delete.</t>
-        </is>
-      </c>
-      <c r="D31" s="23" t="inlineStr">
-        <is>
-          <t>17 deleted files / StaffFilter.java</t>
+      <c r="B31" s="21" t="inlineStr">
+        <is>
+          <t>Có – Tách paymentType (RENTAL/LATE_FEE/EXTENSION) trong Transaction để báo cáo kế toán đúng.</t>
+        </is>
+      </c>
+      <c r="C31" s="21" t="inlineStr">
+        <is>
+          <t>Có – AI đề xuất gộp chung nhưng chọn tách riêng vì yêu cầu dashboard.</t>
+        </is>
+      </c>
+      <c r="D31" s="21" t="inlineStr">
+        <is>
+          <t>PaymentDAO.java / Transaction schema</t>
         </is>
       </c>
     </row>
     <row r="32" ht="86.40000000000001" customHeight="1" s="28">
-      <c r="A32" s="23" t="inlineStr">
+      <c r="A32" s="21" t="inlineStr">
+        <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="B32" s="21" t="inlineStr">
+        <is>
+          <t>Có – IntentClassifier với synonym map và normalize input trước khi match intent chatbot.</t>
+        </is>
+      </c>
+      <c r="C32" s="21" t="inlineStr">
+        <is>
+          <t>Có – AI dùng keyword match đơn giản, bổ sung normalize và synonym để tăng độ chính xác.</t>
+        </is>
+      </c>
+      <c r="D32" s="21" t="inlineStr">
+        <is>
+          <t>ChatbotServlet.java / IntentClassifier.java</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="86.40000000000001" customHeight="1" s="28">
+      <c r="A33" s="21" t="inlineStr">
         <is>
           <t>006</t>
         </is>
       </c>
-      <c r="B32" s="23" t="inlineStr">
-        <is>
-          <t>Có – Phát hiện SyntaxError trong Python script do f-string lồng nháy kép, refactor thành file .py riêng.</t>
-        </is>
-      </c>
-      <c r="C32" s="23" t="inlineStr">
-        <is>
-          <t>Có – Script chạy thành công tạo ra file docx 120 H4 headings.</t>
-        </is>
-      </c>
-      <c r="D32" s="23" t="inlineStr">
-        <is>
-          <t>generate_sds.py (deleted) / MotoRental_SDS_final.docx</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="86.40000000000001" customHeight="1" s="28">
-      <c r="A33" s="23" t="inlineStr">
-        <is>
-          <t>008</t>
-        </is>
-      </c>
-      <c r="B33" s="23" t="inlineStr">
-        <is>
-          <t>Có – Cross-reference SDS với source code, phát hiện DashboardServlet chưa tồn tại, thêm disclaimer.</t>
-        </is>
-      </c>
-      <c r="C33" s="23" t="inlineStr">
-        <is>
-          <t>Có – AI flagged class chưa implement, quyết định ghi chú thay vì xóa.</t>
-        </is>
-      </c>
-      <c r="D33" s="23" t="inlineStr">
-        <is>
-          <t>BookingDAO.java / FeedbackDAO.java / MotoRental_SDS_final.docx</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="115.2" customHeight="1" s="28"/>
+      <c r="B33" s="21" t="inlineStr">
+        <is>
+          <t>Có – Thêm applicableTo flag vào Promotion và update VoucherDAO nhận param bookingType.</t>
+        </is>
+      </c>
+      <c r="C33" s="21" t="inlineStr">
+        <is>
+          <t>Có – Voucher không phân biệt NEW_BOOKING vs EXTENSION gây áp sai discount.</t>
+        </is>
+      </c>
+      <c r="D33" s="21" t="inlineStr">
+        <is>
+          <t>VoucherDAO.java / PromotionServlet.java</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="115.2" customHeight="1" s="28">
+      <c r="A34" s="21" t="inlineStr">
+        <is>
+          <t>007</t>
+        </is>
+      </c>
+      <c r="B34" s="21" t="inlineStr">
+        <is>
+          <t>Có – PaymentExpiryJob server-side thay vì client poll để auto-expire Transaction PENDING.</t>
+        </is>
+      </c>
+      <c r="C34" s="21" t="inlineStr">
+        <is>
+          <t>Có – Client poll không tin cậy nếu đóng tab, cần background job.</t>
+        </is>
+      </c>
+      <c r="D34" s="21" t="inlineStr">
+        <is>
+          <t>PaymentExpiryJob.java / CheckPaymentStatusServlet.java</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:D1"/>

</xml_diff>